<commit_message>
strip residual urls from amerix file (2 rows)
</commit_message>
<xml_diff>
--- a/Topic Relevant Comments/Kenya/Amerix_A Woman Cant Love a Man.xlsx
+++ b/Topic Relevant Comments/Kenya/Amerix_A Woman Cant Love a Man.xlsx
@@ -97,7 +97,7 @@
     <t>You are waffling from the bottom barrel preposterousness of asininity A woman is a core emotionality entity hence more propensity to love more than men A man is a core rationality entity fumbles once oscillates towards heightened emotionality Hence a woman loves A man leads</t>
   </si>
   <si>
-    <t>hawa wanaume wakose tu kulearn lkn wasiguze murima https://t.co/3pdOwltRNO</t>
+    <t>hawa wanaume wakose tu kulearn lkn wasiguze murima</t>
   </si>
   <si>
     <t>Man loves money, money can't love back. It can only be attracted.</t>
@@ -280,7 +280,7 @@
     <t>Mwalimu oozing wisdom like Solomon. Time for toxic women to learn and protect their children from their bad habits</t>
   </si>
   <si>
-    <t>Titus 2:4 KJV [4] that they may teach the young women to be sober, to love their husbands, to love their children, https://t.co/Rf2v1ZcIqe</t>
+    <t>Titus 2:4 KJV [4] that they may teach the young women to be sober, to love their husbands, to love their children,</t>
   </si>
   <si>
     <t>All the men agreeing to this</t>

</xml_diff>